<commit_message>
Update thickness_table_all9.xlsx with 0.005cm and 2 cores setup
</commit_message>
<xml_diff>
--- a/thickness_table_all9.xlsx
+++ b/thickness_table_all9.xlsx
@@ -481,42 +481,42 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
+          <t>0.005, 0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
+          <t>0.005, 0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
+          <t>0.005, 0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
+          <t>0.005, 0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
+          <t>0.005, 0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
+          <t>0.005, 0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
+          <t>0.005, 0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
+          <t>0.005, 0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
         </is>
       </c>
     </row>
@@ -526,42 +526,42 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
+          <t>0.005, 0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
+          <t>0.005, 0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
+          <t>0.005, 0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
+          <t>0.005, 0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
+          <t>0.005, 0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
+          <t>0.005, 0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
+          <t>0.005, 0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
+          <t>0.005, 0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
         </is>
       </c>
     </row>
@@ -571,42 +571,42 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
+          <t>0.005, 0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
+          <t>0.005, 0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
+          <t>0.005, 0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
+          <t>0.005, 0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
+          <t>0.005, 0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
+          <t>0.005, 0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
+          <t>0.005, 0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
+          <t>0.005, 0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
         </is>
       </c>
     </row>
@@ -616,42 +616,42 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
+          <t>0.005, 0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
+          <t>0.005, 0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
+          <t>0.005, 0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
+          <t>0.005, 0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
+          <t>0.005, 0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
+          <t>0.005, 0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
+          <t>0.005, 0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
+          <t>0.005, 0.1, 0.3, 0.5, 0.8, 1.0, 1.5, 2.0, 2.5, 3.0</t>
         </is>
       </c>
     </row>

</xml_diff>